<commit_message>
Add BOG re-liquefaction ideal-work derivation (distinct from fresh-feed calc)
BOG (boil-off gas) is already at ~20.3 K and near-equilibrium para fraction
when it evaporates off the liquid, so re-liquefying it skips both the
sensible-cooling and ortho-para-conversion terms that fresh ambient feed gas
needs -- only the condensation exergy applies. Works out to ~1.71 kWh/kg,
roughly half of fresh-feed liquefaction's 3.3-3.9 kWh/kg, since condensation
is only about 41% of fresh gas's total entropy drop.

Flags two gaps this excludes: real compression work to route low-pressure
BOG into the liquefaction cycle (KHI's ejector/compressor, no SEC
disclosed), and BOG re-liquefaction's unknown real exergetic efficiency.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ae2GGbSYYxRTgFhGrUjGHu
</commit_message>
<xml_diff>
--- a/data/lh2-database.xlsx
+++ b/data/lh2-database.xlsx
@@ -721,7 +721,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1828,6 +1828,55 @@
       <c r="K23" t="inlineStr">
         <is>
           <t>derived: eff = ideal/actual; fairer basis since KHI's process includes O-P conversion (reply Q6/Q7); KHI did not confirm the feed-pressure basis for its 8-9 kWh/kg figure, so both ranges are upper-bound estimates -- a pressurised feed (e.g. this project's 30 barg assumption) implies a lower true ideal-work baseline and therefore a lower true efficiency than shown here</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>liquefaction</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>liquefier</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>theoretical_min_specific_work_bog_reliquefaction</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1.71</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>kWh/kg</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>condensation-only exergy: saturated H2 vapor at NBP (~20.3K) -&gt; saturated liquid at NBP, vs 300K ambient dead state</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>doe-2009-h2-liquefaction-energy</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>ASSUMPTION</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>derived from the same exergy formula/constants as theoretical_min_specific_work_normal/_para, but excluding the sensible-cooling and O-P-conversion terms since BOG starts already cold and near-equilibrium para fraction; excludes any real compression work to route low-pressure BOG into the liquefaction cycle (KHI reply Q3/Q14 ejector/compressor, no separate SEC disclosed)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add regulatory-compliance table to database (mostly gap-flagged)
No dedicated regulatory/permitting coverage existed in the repo before this.
Added data/properties/regulatory-compliance.csv with 9 rows: 2 cited to KHI
(permitting approach Q12, safety separation distance Q36), 7 tagged
needs-source (IMO tank-type classification, IGC/IGF Code, classification
society approval, plant/terminal design codes, carbon-border exposure) --
placeholders only, no fabricated values. Wired into build_db_workbook.py,
tests/test_data_tables.py, and data/README.md with an explicit Known
caveats entry flagging this as unresearched.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KJgheh8pyPfN2k2uFDbHtb
</commit_message>
<xml_diff>
--- a/data/lh2-database.xlsx
+++ b/data/lh2-database.xlsx
@@ -1,20 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="references" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="liquefaction" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="terminals" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="regas" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="lh2_properties" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="lh2_carriers" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="cost_stack" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="chain_energy_defaults" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="references" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="liquefaction" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="terminals" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lh2_properties" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="regulatory_compliance" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="lh2_carriers" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="cost_stack" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="chain_energy_defaults" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3278,7 +3279,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K18"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3341,39 +3342,35 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>commercial_carrier</t>
+          <t>liquefaction_plant</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>cargo_capacity</t>
+          <t>permitting_approach</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>160000</t>
-        </is>
-      </c>
-      <c r="E2" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
+          <t>Design/permit per applicable local laws &amp; regulations; novel (uncovered) items go through a special evaluation committee</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr"/>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>commercial-scale target vessel</t>
+          <t>Japan project experience</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>kawasaki-2026-supplemental</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -3383,46 +3380,42 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>160000 m3/ship on KHI cost-basis slide</t>
+          <t>KHI reply Q12 (rev0331/GHSB20260406, supersedes reply0304). Outside Japan: KHI states only that a 'similar approach' is expected, 'subject to each country's regulatory regime' -- no non-Japan regime confirmed</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>commercial_carrier</t>
+          <t>liquefaction_plant</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>service_speed</t>
+          <t>carbon_intensity_disclosure</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>29.6</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>km/h</t>
-        </is>
-      </c>
+          <t>Feasibility Study necessary; carbon intensity and cost vary with plant size</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr"/>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>design velocity</t>
+          <t>with RE supply</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>kawasaki-2026-supplemental</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -3432,46 +3425,42 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>approx 16 knots</t>
+          <t>KHI reply Q11. Relevant to future carbon-reporting/CBAM-style compliance -- not itself a regulation, but the input KHI ties to one</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>commercial_carrier</t>
+          <t>shipping_carrier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>fleet_count</t>
+          <t>safety_separation_distance</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>ship</t>
-        </is>
-      </c>
+          <t>Significantly larger safety separation distances required vs liquid ammonia (no absolute distance disclosed)</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr"/>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>Base 2.5B Nm3/y</t>
+          <t>qualitative KHI position</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>kawasaki-2026-supplemental</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -3481,657 +3470,229 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>2 ships at Base scale</t>
+          <t>KHI reply additional Q36. LH2 classified as a non-toxic, flammable high-pressure gas</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>commercial_carrier</t>
+          <t>shipping_carrier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>fleet_count</t>
-        </is>
-      </c>
-      <c r="D5" t="inlineStr">
-        <is>
-          <t>8</t>
-        </is>
-      </c>
-      <c r="E5" t="inlineStr">
-        <is>
-          <t>ship</t>
-        </is>
-      </c>
+          <t>imo_tank_type_classification</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="inlineStr"/>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Large 10B Nm3/y</t>
-        </is>
-      </c>
-      <c r="I5" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-supplemental</t>
-        </is>
-      </c>
+          <t>160,000 m3 commercial vessel</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr"/>
       <c r="J5" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>8 ships at Large scale</t>
+          <t>Not confirmed by KHI or any classification society in-repo. IMO Type A/B/C is an LNG taxonomy discussed generically by RSER 2026 and JMSE 2025 (docs/comparison/khi-vs-literature-lh2-comparison.md Sec.2, Sec.6); no source assigns an IMO type to an LH2 carrier specifically</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>carrier_40k</t>
+          <t>shipping_carrier</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>cargo_capacity</t>
-        </is>
-      </c>
-      <c r="D6" t="inlineStr">
-        <is>
-          <t>40000</t>
-        </is>
-      </c>
-      <c r="E6" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
+          <t>applicable_code_or_standard</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr"/>
+      <c r="E6" t="inlineStr"/>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>vessel under construction</t>
-        </is>
-      </c>
-      <c r="I6" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
+          <t>hydrogen-fuelled / hydrogen-carrying ships</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr"/>
       <c r="J6" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>KHI reply Q29; same tank tech as Suiso Frontier, no major issues</t>
+          <t>IGC Code, IGF Code, and any IMO interim guidelines for LH2 carriers not yet sourced in this repo</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>suiso_frontier</t>
+          <t>shipping_carrier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>cargo_capacity</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>1250</t>
-        </is>
-      </c>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>m3</t>
-        </is>
-      </c>
+          <t>classification_society_approval</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr"/>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>demonstration vessel</t>
-        </is>
-      </c>
-      <c r="I7" t="inlineStr">
-        <is>
-          <t>kawasaki-hydrogen-activities</t>
-        </is>
-      </c>
+          <t>class approval / approval-in-principle</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr"/>
       <c r="J7" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>first LH2 carrier; tank tech basis for scale-up</t>
+          <t>No DNV, ClassNK, Lloyd's Register, or ABS rule set or AiP for LH2 carriers cited in-repo</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>carrier</t>
+          <t>liquefaction_plant</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>bog_management</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>BOG used as propulsion fuel</t>
-        </is>
-      </c>
+          <t>applicable_code_or_standard</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>dual-fuel engine (in development)</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
+          <t>plant design/safety code</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>KHI reply Q23/Q32; no onboard reliquefaction</t>
+          <t>No liquefaction-plant code (e.g. national high-pressure gas safety law, NFPA 2, ISO hydrogen standards) sourced in-repo beyond KHI's qualitative Q12 answer above</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>carrier</t>
+          <t>terminal</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>fuel_gas_consumption_rate</t>
-        </is>
-      </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>equal to BOR</t>
-        </is>
-      </c>
+          <t>applicable_code_or_standard</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>only cargo-tank BOG used as fuel</t>
-        </is>
-      </c>
-      <c r="I9" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
+          <t>export/import terminal siting &amp; process safety</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr"/>
       <c r="J9" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>KHI reply Q23; fuel-gas (H2) consumption rate = BOR</t>
+          <t>Exclusion-zone, siting, and process-safety standards for LH2 terminals not yet sourced</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>shipping</t>
+          <t>regulatory</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>carrier</t>
+          <t>chain</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>onboard_reliquefaction</t>
-        </is>
-      </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>not adopted</t>
-        </is>
-      </c>
+          <t>ghg_carbon_border_exposure</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>too much energy + space</t>
-        </is>
-      </c>
-      <c r="I10" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
+          <t>e.g. CBAM-style mechanisms on delivered H2/derivatives</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>KHI reply Q33</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B11" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C11" t="inlineStr">
-        <is>
-          <t>filling_ratio_restriction</t>
-        </is>
-      </c>
-      <c r="D11" t="inlineStr">
-        <is>
-          <t>none</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr">
-        <is>
-          <t>no sloshing impact on BOG</t>
-        </is>
-      </c>
-      <c r="I11" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J11" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K11" t="inlineStr">
-        <is>
-          <t>KHI reply Q20</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B12" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C12" t="inlineStr">
-        <is>
-          <t>max_sailing_distance_limit</t>
-        </is>
-      </c>
-      <c r="D12" t="inlineStr">
-        <is>
-          <t>limited by MGO fuel tank</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr"/>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr">
-        <is>
-          <t>not limited by BOG</t>
-        </is>
-      </c>
-      <c r="I12" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J12" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K12" t="inlineStr">
-        <is>
-          <t>KHI reply Q21</t>
-        </is>
-      </c>
-    </row>
-    <row r="13">
-      <c r="A13" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B13" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>mgo_only_pressure_holding</t>
-        </is>
-      </c>
-      <c r="D13" t="inlineStr">
-        <is>
-          <t>several days within MARVS</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr">
-        <is>
-          <t>100% MGO regime</t>
-        </is>
-      </c>
-      <c r="I13" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J13" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K13" t="inlineStr">
-        <is>
-          <t>KHI reply Q26; GCU burns excess BOG above MARVS</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B14" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr">
-        <is>
-          <t>load_unload_duration</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr">
-        <is>
-          <t>day</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
-      </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>1.5</t>
-        </is>
-      </c>
-      <c r="H14" t="inlineStr">
-        <is>
-          <t>per vessel call</t>
-        </is>
-      </c>
-      <c r="I14" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J14" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K14" t="inlineStr">
-        <is>
-          <t>KHI reply Q27; varies with terminal</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>shipyard</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>KHI Sakaide Shipyard</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr">
-        <is>
-          <t>construction location</t>
-        </is>
-      </c>
-      <c r="I15" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J15" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K15" t="inlineStr">
-        <is>
-          <t>KHI reply Q28; lead time longer than LNG carriers</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>scale_up_challenge</t>
-        </is>
-      </c>
-      <c r="D16" t="inlineStr">
-        <is>
-          <t>cargo tank manufacturability</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr">
-        <is>
-          <t>toward 160000 m3</t>
-        </is>
-      </c>
-      <c r="I16" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J16" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K16" t="inlineStr">
-        <is>
-          <t>KHI reply Q29</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B17" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C17" t="inlineStr">
-        <is>
-          <t>capex_vs_lng</t>
-        </is>
-      </c>
-      <c r="D17" t="inlineStr">
-        <is>
-          <t>significantly higher</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr"/>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr">
-        <is>
-          <t>same-size LNG carrier basis</t>
-        </is>
-      </c>
-      <c r="I17" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J17" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K17" t="inlineStr">
-        <is>
-          <t>KHI reply Q30/Q31; double-wall tanks/piping, limited suppliers</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>shipping</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C18" t="inlineStr">
-        <is>
-          <t>newbuild_cost</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>USD/ship</t>
-        </is>
-      </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr">
-        <is>
-          <t>160000 m3 commercial vessel</t>
-        </is>
-      </c>
-      <c r="I18" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J18" t="inlineStr">
-        <is>
-          <t>needs-source</t>
-        </is>
-      </c>
-      <c r="K18" t="inlineStr">
-        <is>
-          <t>NOT disclosed by KHI (reply Q31); premium over LNG carrier only qualitative</t>
+          <t>No carbon-border or emissions-reporting regime applicable to the LH2 chain has been researched yet</t>
         </is>
       </c>
     </row>
@@ -4146,7 +3707,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4209,39 +3770,39 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>production</t>
+          <t>commercial_carrier</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>cargo_capacity</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>10.1</t>
+          <t>160000</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>commercial-scale target vessel</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-supplemental</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -4251,46 +3812,46 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>IAE Gigaton WS WHTC2019 via kawasaki-2026-supplemental; unit inferred (slide unlabelled), ~2019 vintage [needs source: primary]</t>
+          <t>160000 m3/ship on KHI cost-basis slide</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>liquefaction</t>
+          <t>commercial_carrier</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>service_speed</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>10.3</t>
+          <t>29.6</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>km/h</t>
         </is>
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>design velocity</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-supplemental</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -4300,46 +3861,46 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>approx 16 knots</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>loading_terminal</t>
+          <t>commercial_carrier</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>fleet_count</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>5.6</t>
+          <t>2</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>ship</t>
         </is>
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>Base 2.5B Nm3/y</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-supplemental</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -4349,46 +3910,46 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>2 ships at Base scale</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>seaborne_transport</t>
+          <t>commercial_carrier</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>fleet_count</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>4.0</t>
+          <t>8</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>ship</t>
         </is>
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>Large 10B Nm3/y</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-supplemental</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -4398,46 +3959,46 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>8 ships at Large scale</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>receiving_terminal</t>
+          <t>carrier_40k</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>cargo_capacity</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>6.3</t>
+          <t>40000</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>vessel under construction</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -4447,46 +4008,46 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q29; same tank tech as Suiso Frontier, no major issues</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>dehydrogenation</t>
+          <t>suiso_frontier</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>cargo_capacity</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>0.0</t>
+          <t>1250</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>m3</t>
         </is>
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>demonstration vessel</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-hydrogen-activities</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -4496,46 +4057,42 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>zero for LH2 (no reconversion step); IAE via KHI [needs source: primary]</t>
+          <t>first LH2 carrier; tank tech basis for scale-up</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>bog_management</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="E8" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>BOG used as propulsion fuel</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr"/>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>dual-fuel engine (in development)</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -4545,46 +4102,42 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q23/Q32; no onboard reliquefaction</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>fuel_gas_consumption_rate</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>37.6</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>equal to BOR</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr"/>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
-          <t>LH2 Base</t>
+          <t>only cargo-tank BOG used as fuel</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -4594,46 +4147,42 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>sum of LH2 Base components; reconciliation check</t>
+          <t>KHI reply Q23; fuel-gas (H2) consumption rate = BOR</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>production</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>onboard_reliquefaction</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>10.1</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>not adopted</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr"/>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>too much energy + space</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -4643,46 +4192,42 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q33</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>liquefaction</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>filling_ratio_restriction</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="E11" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>none</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr"/>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>no sloshing impact on BOG</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -4692,46 +4237,42 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q20</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>loading_terminal</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>max_sailing_distance_limit</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>1.9</t>
-        </is>
-      </c>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>limited by MGO fuel tank</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>not limited by BOG</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -4741,46 +4282,42 @@
       </c>
       <c r="K12" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q21</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>seaborne_transport</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>mgo_only_pressure_holding</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>4.0</t>
-        </is>
-      </c>
-      <c r="E13" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>several days within MARVS</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr"/>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>100% MGO regime</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -4790,46 +4327,50 @@
       </c>
       <c r="K13" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q26; GCU burns excess BOG above MARVS</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>receiving_terminal</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D14" t="inlineStr">
-        <is>
-          <t>3.4</t>
-        </is>
-      </c>
+          <t>load_unload_duration</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+          <t>day</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>1.5</t>
+        </is>
+      </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>per vessel call</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -4839,46 +4380,42 @@
       </c>
       <c r="K14" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q27; varies with terminal</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>dehydrogenation</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>shipyard</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>KHI Sakaide Shipyard</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr"/>
       <c r="F15" t="inlineStr"/>
       <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>construction location</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -4888,46 +4425,42 @@
       </c>
       <c r="K15" t="inlineStr">
         <is>
-          <t>zero for LH2 (no reconversion step); IAE via KHI [needs source: primary]</t>
+          <t>KHI reply Q28; lead time longer than LNG carriers</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>other</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>scale_up_challenge</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>cargo tank manufacturability</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr"/>
       <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>toward 160000 m3</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -4937,46 +4470,42 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+          <t>KHI reply Q29</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>TOTAL</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>supply_cost</t>
+          <t>capex_vs_lng</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>30.7</t>
-        </is>
-      </c>
-      <c r="E17" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
+          <t>significantly higher</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr"/>
       <c r="F17" t="inlineStr"/>
       <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
-          <t>LH2 Large</t>
+          <t>same-size LNG carrier basis</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -4986,579 +4515,52 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>sum of LH2 Large components; reconciliation check</t>
+          <t>KHI reply Q30/Q31; double-wall tanks/piping, limited suppliers</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>cost</t>
+          <t>shipping</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>production</t>
+          <t>carrier</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D18" t="inlineStr">
-        <is>
-          <t>9.3</t>
-        </is>
-      </c>
+          <t>newbuild_cost</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
-          <t>JPY/Nm3</t>
+          <t>USD/ship</t>
         </is>
       </c>
       <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
-          <t>LH2 Tech</t>
+          <t>160000 m3 commercial vessel</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>iae-2019-gigaton</t>
+          <t>kawasaki-2026-questionnaire</t>
         </is>
       </c>
       <c r="J18" t="inlineStr">
         <is>
-          <t>cited</t>
+          <t>needs-source</t>
         </is>
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B19" t="inlineStr">
-        <is>
-          <t>liquefaction</t>
-        </is>
-      </c>
-      <c r="C19" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D19" t="inlineStr">
-        <is>
-          <t>8.6</t>
-        </is>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I19" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J19" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K19" t="inlineStr">
-        <is>
-          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>loading_terminal</t>
-        </is>
-      </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D20" t="inlineStr">
-        <is>
-          <t>1.8</t>
-        </is>
-      </c>
-      <c r="E20" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I20" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J20" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K20" t="inlineStr">
-        <is>
-          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B21" t="inlineStr">
-        <is>
-          <t>seaborne_transport</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr">
-        <is>
-          <t>2.3</t>
-        </is>
-      </c>
-      <c r="E21" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I21" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J21" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K21" t="inlineStr">
-        <is>
-          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B22" t="inlineStr">
-        <is>
-          <t>receiving_terminal</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D22" t="inlineStr">
-        <is>
-          <t>2.8</t>
-        </is>
-      </c>
-      <c r="E22" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I22" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J22" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K22" t="inlineStr">
-        <is>
-          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B23" t="inlineStr">
-        <is>
-          <t>dehydrogenation</t>
-        </is>
-      </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D23" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
-      </c>
-      <c r="E23" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I23" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J23" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K23" t="inlineStr">
-        <is>
-          <t>zero for LH2 (no reconversion step); IAE via KHI [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B24" t="inlineStr">
-        <is>
-          <t>other</t>
-        </is>
-      </c>
-      <c r="C24" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D24" t="inlineStr">
-        <is>
-          <t>1.3</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I24" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J24" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K24" t="inlineStr">
-        <is>
-          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B25" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="C25" t="inlineStr">
-        <is>
-          <t>supply_cost</t>
-        </is>
-      </c>
-      <c r="D25" t="inlineStr">
-        <is>
-          <t>26.1</t>
-        </is>
-      </c>
-      <c r="E25" t="inlineStr">
-        <is>
-          <t>JPY/Nm3</t>
-        </is>
-      </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr">
-        <is>
-          <t>LH2 Tech</t>
-        </is>
-      </c>
-      <c r="I25" t="inlineStr">
-        <is>
-          <t>iae-2019-gigaton</t>
-        </is>
-      </c>
-      <c r="J25" t="inlineStr">
-        <is>
-          <t>cited</t>
-        </is>
-      </c>
-      <c r="K25" t="inlineStr">
-        <is>
-          <t>sum of LH2 Tech components; reconciliation check</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B26" t="inlineStr">
-        <is>
-          <t>liquefaction</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>capex_specific</t>
-        </is>
-      </c>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr">
-        <is>
-          <t>USD/kg</t>
-        </is>
-      </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
-      <c r="H26" t="inlineStr">
-        <is>
-          <t>reasonable-size plant</t>
-        </is>
-      </c>
-      <c r="I26" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J26" t="inlineStr">
-        <is>
-          <t>needs-source</t>
-        </is>
-      </c>
-      <c r="K26" t="inlineStr">
-        <is>
-          <t>NOT disclosed by KHI (reply Q8): Feasibility Study necessary</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B27" t="inlineStr">
-        <is>
-          <t>liquefaction</t>
-        </is>
-      </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>opex_specific</t>
-        </is>
-      </c>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr">
-        <is>
-          <t>USD/kg</t>
-        </is>
-      </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
-      <c r="H27" t="inlineStr">
-        <is>
-          <t>reasonable-size plant</t>
-        </is>
-      </c>
-      <c r="I27" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J27" t="inlineStr">
-        <is>
-          <t>needs-source</t>
-        </is>
-      </c>
-      <c r="K27" t="inlineStr">
-        <is>
-          <t>NOT disclosed by KHI (reply Q9): Feasibility Study necessary</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B28" t="inlineStr">
-        <is>
-          <t>receiving_terminal</t>
-        </is>
-      </c>
-      <c r="C28" t="inlineStr">
-        <is>
-          <t>regas_capex_specific</t>
-        </is>
-      </c>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr">
-        <is>
-          <t>USD/kg</t>
-        </is>
-      </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
-      <c r="H28" t="inlineStr">
-        <is>
-          <t>reasonable-size terminal</t>
-        </is>
-      </c>
-      <c r="I28" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J28" t="inlineStr">
-        <is>
-          <t>needs-source</t>
-        </is>
-      </c>
-      <c r="K28" t="inlineStr">
-        <is>
-          <t>not separately disclosed by KHI; only IAE aggregate available</t>
-        </is>
-      </c>
-    </row>
-    <row r="29">
-      <c r="A29" t="inlineStr">
-        <is>
-          <t>cost</t>
-        </is>
-      </c>
-      <c r="B29" t="inlineStr">
-        <is>
-          <t>carrier</t>
-        </is>
-      </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>newbuild_cost</t>
-        </is>
-      </c>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr">
-        <is>
-          <t>USD/ship</t>
-        </is>
-      </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>160000 m3 vessel</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>kawasaki-2026-questionnaire</t>
-        </is>
-      </c>
-      <c r="J29" t="inlineStr">
-        <is>
-          <t>needs-source</t>
-        </is>
-      </c>
-      <c r="K29" t="inlineStr">
-        <is>
-          <t>NOT disclosed by KHI (reply Q31)</t>
+          <t>NOT disclosed by KHI (reply Q31); premium over LNG carrier only qualitative</t>
         </is>
       </c>
     </row>
@@ -5573,6 +4575,1433 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:K29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>segment</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>component</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>high</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>basis</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>source_id</t>
+        </is>
+      </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>tag</t>
+        </is>
+      </c>
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr"/>
+      <c r="G2" t="inlineStr"/>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>IAE Gigaton WS WHTC2019 via kawasaki-2026-supplemental; unit inferred (slide unlabelled), ~2019 vintage [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>liquefaction</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>10.3</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr"/>
+      <c r="G3" t="inlineStr"/>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>loading_terminal</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>5.6</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K4" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>seaborne_transport</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>receiving_terminal</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>6.3</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr"/>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K6" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>dehydrogenation</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr"/>
+      <c r="G7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>zero for LH2 (no reconversion step); IAE via KHI [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>37.6</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr"/>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>LH2 Base</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>sum of LH2 Base components; reconciliation check</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>10.1</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>liquefaction</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr"/>
+      <c r="G11" t="inlineStr"/>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>loading_terminal</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>1.9</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr"/>
+      <c r="G12" t="inlineStr"/>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>seaborne_transport</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>4.0</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>receiving_terminal</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>3.4</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr"/>
+      <c r="G14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>dehydrogenation</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t>zero for LH2 (no reconversion step); IAE via KHI [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr"/>
+      <c r="G16" t="inlineStr"/>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t>IAE via KHI; unit inferred JPY/Nm3 ~2019 [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>30.7</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr"/>
+      <c r="G17" t="inlineStr"/>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>LH2 Large</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t>sum of LH2 Large components; reconciliation check</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>production</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>9.3</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
+      <c r="G18" t="inlineStr"/>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>liquefaction</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>8.6</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr"/>
+      <c r="G19" t="inlineStr"/>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>loading_terminal</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>1.8</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>seaborne_transport</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>2.3</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr"/>
+      <c r="G21" t="inlineStr"/>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>receiving_terminal</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>2.8</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr"/>
+      <c r="G22" t="inlineStr"/>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>dehydrogenation</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr"/>
+      <c r="G23" t="inlineStr"/>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t>zero for LH2 (no reconversion step); IAE via KHI [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>1.3</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr"/>
+      <c r="G24" t="inlineStr"/>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t>IAE via KHI; technological-progress case [needs source: primary]</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>supply_cost</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>26.1</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>JPY/Nm3</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr"/>
+      <c r="G25" t="inlineStr"/>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>LH2 Tech</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>iae-2019-gigaton</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>cited</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>sum of LH2 Tech components; reconciliation check</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>liquefaction</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>capex_specific</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr"/>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>USD/kg</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr"/>
+      <c r="G26" t="inlineStr"/>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>reasonable-size plant</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>kawasaki-2026-questionnaire</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>needs-source</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>NOT disclosed by KHI (reply Q8): Feasibility Study necessary</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>liquefaction</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>opex_specific</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr"/>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>USD/kg</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr"/>
+      <c r="G27" t="inlineStr"/>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>reasonable-size plant</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>kawasaki-2026-questionnaire</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>needs-source</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>NOT disclosed by KHI (reply Q9): Feasibility Study necessary</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>receiving_terminal</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>regas_capex_specific</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr"/>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>USD/kg</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr"/>
+      <c r="G28" t="inlineStr"/>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>reasonable-size terminal</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>kawasaki-2026-questionnaire</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>needs-source</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>not separately disclosed by KHI; only IAE aggregate available</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>cost</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>carrier</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>newbuild_cost</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>USD/ship</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr"/>
+      <c r="G29" t="inlineStr"/>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>160000 m3 vessel</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>kawasaki-2026-questionnaire</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>needs-source</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>NOT disclosed by KHI (reply Q31)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>

</xml_diff>